<commit_message>
output xlsx file formate change
</commit_message>
<xml_diff>
--- a/output/test/book-output.xlsx
+++ b/output/test/book-output.xlsx
@@ -27,7 +27,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -40,8 +40,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,10 +63,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -433,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -476,6 +480,175 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>প্রতিবেশীর হক্ক আদায়কারী</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>প্রতিবেশীর হক্ক আদায়কারী</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>&lt;div class="page-text"&gt;&lt;br&gt;প্রতিবেশী আত্মীয় হোক অথবা অনাত্মীয়, মুসলিম হোক অথবা অমুসলিম সর্বাবস্থায় সাধ্যানুযায়ী তাদের সাহায্য-সহায়তা করা ও তাদের খবরাখবর নেয়া জরুরী।&lt;br&gt;&lt;br&gt;
+যারা প্রতিবেশীকে কষ্ট দেয়, তারা জান্নাতে যাবে না। এদের ব্যাপারে রাসূলুল্লাহ (ﷺ) কসম করে বলেছেন, যেসব কারণে মানুষ জান্নাতে যাবে না, প্রতিবেশীকে কষ্ট প্রদানকারী তার অন্যতম। আল্লাহ তাআলা বলেন,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;وَاعْبُدُوا اللهَ وَلَا تُشْرِكُوا بِهِ شَيْئًا وَبِالْوَالِدَيْنِ إِحْسَانًا وَبِذِي الْقُرْبَى وَالْيَتَامَى وَالْمَسَاكِينِ وَالْجَارِ ذِي الْقُرْبَى وَالْجَارِ الْجُنُبِ وَالصَّاحِبِ بِالْجَنْبِ وَابْنِ السَّبِيلِ وَمَا مَلَكَتْ أَيْمَانُكُمْ إِنَّ اللهَ لَا يُحِبُّ مَنْ كَانَ مُخْتَالاً فَخُورًا.&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+'তোমরা আল্লাহর ইবাদত করো, তাঁর সাথে কাউকে শরীক করো না এবং পিতা-মাতা, আত্মীয়-স্বজন, ইয়াতীম, অভাবগ্রস্ত, নিকট প্রতিবেশী, দূর প্রতিবেশী, সঙ্গী-সাথী, মুসাফির ও তোমাদের অধিকারভুক্ত দাস- দাসীদের প্রতি সদ্ব্যবহার করো। নিশ্চয়ই আল্লাহ দাম্ভিক অহংকারীকে পছন্দ করেন না' (নিসা, ৩৬)।&lt;br&gt;&lt;br&gt;
+এই আয়াতে আল্লাহ তাআলা প্রতিবেশীর হক্ক উল্লেখ করেছেন এবং যারা প্রতিবেশীর সাথে ভালো ব্যবহার করে না, তাদেরকে অহংকারী ও দাম্ভিক বলেছেন।&lt;br&gt;&lt;br&gt;
+পিতামাতার সাথে ভালো ব্যবহারের নির্দেশ দানের পাশাপাশি নিকটবর্তী ও দূরবর্তী প্রতিবেশী এবং দাস-দাসীর সাথেও উত্তম ব্যবহার করার নির্দেশ দেওয়া হয়েছে উপরোক্ত আয়াতে। কেননা প্রতিবেশী ও দাস- দাসীরাই মানুষের বিপদে-আপদে সর্বাগ্রে এগিয়ে আসে। তাই এসব লোকের সাথে ভালো আচরণ করা আদর্শ পুরুষের কর্তব্য।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ اللهِ قَالَ: قَالَ رَسُولُ اللهِ  : «واللهِ لَا يُؤْمِنُ، وَاللَّهِ لَا يُؤْمِنُ، وَاللَّهِ لَا يُؤْمِنُ قِيلَ : مَنْ يَا رَسُول الله؟ قَالَ الَّذِي لَا يَأْمَنُ جَارُهُ بَوَائِقَهُ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;আবু হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'আল্লাহর কসম! সে ঈমানদার নয়। আল্লাহর কসম! সে ঈমানদার নয়। আল্লাহর কসম! সে ঈমানদার নয়। বলা হলো, হে আল্লাহর রাসূল! সে কে? তিনি বললেন, যার প্রতিবেশী তার অনিষ্টতা হতে নিরাপদ নয়' (ছহীহ বুখারী, হা/৬০১৬; মুসনাদে আহমাদ, হা/৮০৯৭; মিশকাত, হা/৪৯৬২)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَنَسٍ قَالَ: قَالَ رَسُولُ الله الله : «لا يَدْخُلُ الجَنَّةَ مَنْ لَا يَأْمَنُ جَارُهُ بَوَائِقَهُ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আনাস (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, সে ব্যক্তি জান্নাতে প্রবেশ করবে না, যার প্রতিবেশী তার অনিষ্টতা হতে নিরাপদ নয়' (ছহীহ মুসলিম, হা/১৮১; মুসনাদে আহমাদ, হা/৯০৯০; মিশকাত, হা/৪০৬৩)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: قَالَ رَسُولُ اللهِ  : «مَنْ كَانَ يُؤْمِنُ بِاللهِ وَالْيَوْمِ الْآخِرِ فَلَا يُؤْذِ جَارَهُ وَمَنْ كَانَ يُؤْمِنُ بِاللَّهِ وَالْيَوْمِ الْآخِرِ فَلْيُكْرِمْ ضَيْفَهُ وَمَنْ كَانَ يُؤْمِنُ بِاللَّهِ وَالْيَوْمِ الْآخِرِ فَلْيَقُلْ خَيْرًا أَوْ لِيَصْمُتْ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবু হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'যে ব্যক্তি আল্লাহ ও পরকালের প্রতি ঈমান রাখে, সে যেন তার প্রতিবেশীকে কষ্ট না দেয়। আর যে ব্যক্তি আল্লাহ ও পরকালের প্রতি ঈমান রাখে, সে যেন তার মেহমানকে সম্মান করে। অনুরূপ যে ব্যক্তি আল্লাহ ও পরকালের প্রতি ঈমান রাখে, সে যেন ভালো কথা বলে অথবা চুপ থাকে' (ছহীহ বুখারী, হা/৬০১৮, ছহীহ মুসলিম, হা/১৮২; মিশকাত, হা/৪২৪৩)।&lt;br&gt;&lt;br&gt;
+উল্লেখিত হাদীছসমূহ হতে বিশেষভাবে প্রতীয়মান হয় যে, প্রতিবেশীর হক অত্যন্ত গুরুত্বপূর্ণ বিষয়। যার সাথে জান্নাত পাওয়ার বিষয়টি সংশ্লিষ্ট। তাই প্রতিবেশীর হক আদায় করে জান্নাতের পথ সুগম করা প্রত্যেক মুমিন নর-নারীর জন্য আবশ্যক।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ عَائِشَةَ وَابْنِ عَمْرَ عَنِ النَّبِي صَلى اللَّهِ ﷺ يَقُولُ : مَا يُوصِينِي بِالْجَارِ حَتَّى ظَنَنْتُ أَنَّهُ سیورت&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আয়েশা ও ইবনু উমার (রাঃ) হতে বর্ণিত, নবী (ﷺ) বলেছেন, 'জিবরীল (আঃ) এসে আমাকে প্রতিবেশীর ব্যাপারে অবিরত উপদেশ দিতে থাকতেন। এমনকি মনে হত যে, হয়ত তিনি প্রতিবেশীকে সম্পদের ওয়ারিশ বানিয়ে দিবেন' (ছহীহ বুখারী, হা/৬০১৪, ছহীহ মুসলিম, হা/৬৮৫৪; মিশকাত, হা/৪৯৬৪)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ لله عَنْ النَّبِيِّ ﷺ قَالَ : يَا نِسَاءَ الْمُسْلِمَاتِ لَا تَحْقِرَنَّ جَارَةُ لِجَارَتِهَا وَلَوْ فِرْسِنَ شَاةٍ.&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবু হুরায়রা (রাঃ) হতে বর্ণিত, নবী (ﷺ) বলেছেন, 'হে মুসলিম মহিলাগণ! কোনো মহিলা তার প্রতিবেশীকে তুচ্ছ মনে করবে না। এমনকি ছাগলের পায়ের ক্ষুর হলেও প্রতিবেশীর নিকট পাঠাতে হবে' (ছহীহ বুখারী, হা/৬০১৭; ছহীহ মুসলিম, হা/২৪২৬; মিশকাত, হা/১৮৯২)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ عَائِشَةَ رَضِيَ اللَّهُ عَنْهَا قُلْتُ: يَا رَسُولَ اللَّهِ إِنَّ لِي جَارَيْنِ فَإِلَى أَيْهِمَا أُهْدِي قَالَ: «إِلَى أَقْرَبِهِمَا مِنْكِ بَابًا».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আয়েশা (রাঃ) হতে বর্ণিত, আমি বললাম, হে আল্লাহর রাসূল! আমার দুটি প্রতিবেশী আছে। এদের মধ্যে কাকে আমি হাদিয়া প্রদান করবো? তিনি বললেন, 'উভয়ের মধ্যে যার বাড়ি তোমার বেশী কাছে তাকে' (ছহীহ বুখারী, হা/২২৫৯; আবূ দাউদ, হা/৫১৫৫; মিশকাত, হা/১৯৩৬)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي ذَرٍّ قَالَ: قَالَ رَسُولُ اللهِ ﷺ : «يَا أَبَا ذَرٍّ إِذَا طَبَخْتَ مَرَقَةً فَأَكْثِرْ مَاءَهَا وَتَعَاهَدْ جِيرَانَكَ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ যার (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'হে আবূ যার! যখন তুমি তরকারী রান্না কর, তখন একটু বেশি পানি দিয়ে ঝোল বেশি করো এবং তোমার প্রতিবেশীর হক্ক পৌঁছে দাও' (ছহীহ মুসলিম, হা/৬৮৫৫, সুনান আদ-দারেমী হা/২১৩২; মিশকাত, হা/১৯৩৭)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ لله أَنَّ رَسُولَ اللهِ ﷺ قَالَ : لا يَمْنَعْ أَحَدُكُمْ جَارَهُ أَنْ يَغْرِزَ خَشَبَةً فِي جداره».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ হুরায়রা (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) বলেছেন, 'এক প্রতিবেশী যেন অপর প্রতিবেশীকে দেওয়ালের সাথে খুঁটি গাড়তে নিষেধ না করে' (ছহীহ বুখারী, হা/২৪৬৩; ছহীহ মুসলিম, হা/৪২১৫; মিশকাত, হা/২৯৬৪)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ عُقْبَةَ بْنِ عَامِرٍ الله قَالَ : قَالَ رَسُولُ اللهِ ﷺ : «أَوَّلُ خَصْمَيْنِ يَوْمَ الْقِيَامَةِ جَارَانِ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+উক্ববা ইবনু আমের (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'কিয়ামতের দিন সর্বপ্রথম ঝগড়াটে দুই প্রতিবেশীর মুকদ্দমা পেশ করা হবে' (আহমাদ হা/১৭৮৩৬; মিশকাত, হা/৫০০০)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنِ ابْنِ عَبَّاسٍ قَالَ: سَمِعْتُ رَسُولَ اللهِ ﷺ يَقُوْلُ : لَيْسَ الْمُؤْمِنُ بِالَّذِي يَشْبَعُ وَجَارُهُ جَائِعٌ إِلَى جَنْبِهِ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আব্দুল্লাহ ইবনু আব্বাস (রাঃ) হতে বর্ণিত, তিনি বলেন, আমি রাসূলুল্লাহ (ﷺ)-কে বলতে শুনেছি, ঐ ব্যক্তি মুমিন নয়, যে উদর পূর্ণ করে খায় আর তার পার্শ্বেই তার প্রতিবেশী ক্ষুধার্ত থাকে' (বায়হাক্বী হা/৩৩৮৯; মিশকাত, হা/৪৯৯১)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: قَالَ رَجُلٌ يَا رَسُوْلَ اللهِ إِنَّ فُلَانَةً تُذْكَرُ مِنْ كَثْرَةِ صَلَاتِهَا وَصِيَامِهَا وَصَدَقَتِهَا غَيْرَ أَنَّهَا تُؤْذِي جِيْرَانَهَا بِلِسَانِهَا قَالَ: هِيَ فِي النَّارِ، قَالَ يَا رَسُولَ اللَّهِ فَإِنَّ فُلَانَةٌ تُذْكَرُ مِنْ قِلَّةِ صِيَامِهَا وَصَدَقَتِهَا وَصَلَاتِهَا وَإِنَّهَا تَصَدَّقُ بِالْأَنْوَارِ مِنْ الْأَقِطِ وَلَا تُؤْذِي بِلِسَانِهَا جِيْرَانَهَا قَالَ: هِيَ فِي الْجَنَّةِ.&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, একদা জনৈক ব্যক্তি বলল, হে আল্লাহর রাসূল! অমুক মহিলা অধিক ছালাত পড়ে, ছিয়াম রাখে এবং দান-ছাদাক্বা করার ব্যাপারে প্রসিদ্ধি লাভ করেছে। তবে সে নিজের মুখের দ্বারা স্বীয় প্রতিবেশীদেরকে কষ্ট দেয়। তিনি বললেন, সে জাহান্নামী। লোকটি আবার বলল, হে আল্লাহর রাসূল! অমুক মহিলা যার সম্পর্কে জনশ্রুতি আছে যে, সে কম ছিয়াম পালন করে, দান-ছাদাক্বাও কম করে এবং ছালাতও কম আদায় করে। তার দানের পরিমাণ হল পনিরের টুকরা বিশেষ। কিন্তু সে নিজের মুখ দ্বারা স্বীয় প্রতিবেশীদেরকে কষ্ট দেয় না। তিনি বললেন, সে জান্নাতী' (আহমাদ হা/৯৯২৬; মিশকাত, হা/৪৯৯২)।&lt;br&gt;&lt;br&gt;
+উপরিউক্ত কুরআনের আয়াত ও হাদীছসমূহ দ্বারা প্রতীয়মান হয় যে, প্রতিবেশীর হক অত্যধিক। তাদের সাথে সদাচরণ করা প্রত্যেক মুমিনের অবশ্য কর্তব্য। তাদের কষ্ট দেওয়া থেকে বিরত থাকাও রাসূলের নির্দেশ। খাদ্য আদান-প্রদান ও উত্তম আচরণের মাধ্যমে তাদের সাথে সুসম্পর্ক বজায় রাখা জরুরী। প্রতিবেশীর হক্ক আদায় না করলে এবং তাদের সাথে ভালো ব্যবহার না করলে জান্নাত পাওয়া কঠিন।&lt;br&gt;&lt;br&gt;&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>পিতামাতার সাথে সদ্ব্যবহারকারী</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>পিতামাতার সাথে সদ্ব্যবহারকারী</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>&lt;div class="page-text"&gt;&lt;br&gt;পিতামাতা আল্লাহর পক্ষ থেকে এক অতুলনীয় নেয়ামত। আল্লাহ তাঁর ইবাদতের পরেই পিতামাতার সাথে সদ্ব্যবহারের নির্দেশ দিয়েছেন। পিতামাতার সাথে সদ্ব্যবহার জান্নাতে যাওয়ার মাধ্যম হিসাবে আল্লাহর রাসূল আলাইহে উল্লেখ করেছেন। পিতামাতাকে পেয়ে তাদের সাথে সদাচরণ করে যে ব্যক্তি জান্নাত লাভ করতে পারল না, তার চেয়ে হতভাগা আর নেই। পিতামাতা অত্যাচারী, অন্যায়কারী, এমনকি বিধর্মী হলেও তাদের সাথে উত্তম ব্যবহার করার জন্য রাসূলুল্লাহ (ﷺ) নির্দেশ দিয়েছেন। পিতামাতার সাথে সদাচরণের নির্দেশ দিয়ে আল্লাহ বলেন,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;وَوَصَّيْنَا الْإِنْسَانَ بِوَالِدَيْهِ حَمَلَتْهُ أُمُّهُ وَهْنًا عَلَى وَهْنٍ وَفِصَالُهُ فِي عَامَيْنِ أَنِ اشْكُرْ لِي وَلِوَالِدَيْكَ إِلَيَّ الْمَصِيرُ).&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+'আ'মি মানুষকে তার পিতামাতার সাথে সদ্ব্যবহার করার নির্দেশ দিয়েছি। তার মা কষ্টের পর কষ্ট করে গর্ভে ধারণ করেছে। একাধারে দুবছর দুধ পান করিয়েছে। অতএব আমার প্রতি ও পিতামাতার প্রতি কৃতজ্ঞ হও। আর আমার নিকটেই তোমাদের ফিরে আসতে হবে' (লুকমান, ১৪)।&lt;br&gt;&lt;br&gt;
+তিনি আরো বলেন,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;وَقَضَى رَبُّكَ أَلَّا تَعْبُدُوا إِلَّا إِيَّاهُ وَبِالْوَالِدَيْنِ إِحْسَانًا إِمَّا يَبْلُغَنَّ عِنْدَكَ الْكِبَرَ أَحَدُهُمَا أَوْ كِلَاهُمَا فَلَا تَقُلْ لَهُمَا أُفٍّ وَلَا تَنْهَرْهُمَا وَقُلْ لَهُمَا قَوْلًا كَرِيمًا وَاخْفِضْ لَهُمَا جَنَاحَ الذُّلِّ مِنَ الرَّحْمَةِ وَقُلْ رَبِّ ارْحَمْهُمَا كَمَا رَبَّيَانِي صَغِيرًا.&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+'তোমার পালনকর্তা নির্দেশ দিচ্ছেন যে, তোমরা, তাকে ছাড়া যেন অন্য কারো ইবাদত না কর। এবং পিতামাতার সাথে সদ্ব্যবহার কর। তাদের মধ্যে কেউ অথবা উভয়ই যদি তোমার জীবদ্দশায় বার্ধক্যে উপনীত হয়, তবে তাদেরকে 'উহ্' শব্দটিও বলবে না এবং তাদেরকে ধমক দিবে না ও তাদের সাথে শিষ্টাচারপূর্ণ কথা বল। তাদের সাথে নম্রভাবে করুণার ডানা অবনত&lt;br&gt;&lt;br&gt;করে দাও এবং বল, হে আমার পালনকর্তা। তাদের উভয়ের প্রতি রহম কর, যেমনভাবে তারা শৈশবে আমাকে লালন-পালন করেছে' (বানী ইসরাঈল, ২৩-২৪)।&lt;br&gt;&lt;br&gt;
+এই আয়াতে আল্লাহ তাঁর ইবাদতের পরেই পিতামাতার সাথে উত্তম আচরণের নির্দেশ দিয়েছেন। (১) সন্তানের কোনো কাজের জন্য পিতামাতা যেন কষ্ট না পায়, সেদিকে লক্ষ্য রাখতে হবে। (২) তাদের কোনো কাজের জন্য তাদেরকে ধমক বা কষ্ট দেওয়া যাবে না। তাদের সাথে উত্তম আচরণ করতে হবে। তাদের সাথে সদা নম্র-ভদ্র ব্যবহার করতে হবে। (৩) বৃদ্ধাবস্থায় তাদের প্রতি দয়ার হাত বাড়িয়ে দিতে হবে। (৪) তাদের মৃত্যুর পরে তাদের জন্য দু'আ করতে হবে। এই আয়াত ব্যতীত আরো অনেক আয়াতে আল্লাহ এভাবে পিতামাতার সাথে সদ্ব্যবহার করা নির্দেশ দিয়েছেন।&lt;br&gt;&lt;br&gt;
+পিতামাতার প্রতি সদাচরণের গুরুত্ব সম্পর্কে হাদীছে এসেছে,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ عَبْدِ اللَّهِ بْنِ عَمْرٍو قال : سَأَلْتُ النَّبِيَّ  : «أَيُّ الْعَمَلِ أَحَبُّ إِلَى اللَّهِ؟ قَالَ: الصَّلَاةُ عَلَى وَقْتِهَا، قَالَ: ثُمَّ أَيُّ؟ قَالَ: ثُمَّ بِرُّ الْوَالِدَيْنِ ، قَالَ : ثُمَّ أَيُّ؟ قَالَ: الْجِهَادُ فِي سَبِيلِ اللَّهِ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আব্দুল্লাহ ইবনু আমর (রাঃ) হতে বর্ণিত, তিনি বলেন, নবী (ﷺ)-কে জিজ্ঞেস করলাম, হে আল্লাহর রাসূল! আল্লাহর নিকট সবচেয়ে পছন্দনীয় আমল কী? তিনি? বললেন, 'সময়মত ছালাত আদায় করা। আবার জিজ্ঞেস করলাম, তারপর কী? তিনি বললেন, তারপর হচ্ছে পিতা-মাতার অনুগত হওয়া। তারপর জিজ্ঞেস করলাম, এরপর কী? তিনি বললেন, আল্লাহর রাস্তায় জিহাদ করা' (ছহীহ বুখারী, হা/৫২৭; ছহীহ মুসলিম, হা/২৬৪; মিশকাত, হা/৫৬৮)।&lt;br&gt;&lt;br&gt;
+এই হাদীছে আল্লাহর নিকট পছন্দনীয় আমল সময়মত ছালাত আদায়ের পরই পিতামাতার সাথে সদাচরণের কথা বলা হয়েছে। এমনকি এতে জিহাদের উপরেও পিতামাতার সাথে সদ্ব্যবহারকে গুরুত্ব দেওয়া হয়েছে। উল্লেখ্য যে, পিতামাতার মধ্যে মায়ের মর্যাদা পিতার চেয়ে তিনগুণ বেশী বলে হাদীছে উল্লেখিত হয়েছে।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ لله قَالَ: «قَالَ رَجُلٌ : يَا رَسُولَ اللهِ مَنْ أَحَقُّ بِحُسْنِ صَحَابَتِي؟ قَالَ: أُمُّكَ قَالَ: ثُمَّ مَنْ؟ قَالَ: أُمُّكَ . قَالَ : ثُمَّ مَنْ؟ قَالَ: أُمُّكَ قَالَ : ثُمَّ مَنْ؟ قَالَ: أَبُوكَ». وَفِي رِوَايَةٍ قَالَ: «أُمَّكَ، ثُمَّ أُمَّكَ، ثُمَّ أُمَّكَ، ثُمَّ أَبَاكَ، ثُمَّ أَدْنَاكَ أَدْنَاكَ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবু হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, এক ব্যক্তি বলল, হে আল্লাহর রাসূল! আমার নিকট সর্বাপেক্ষা অধিক ভালো আচরণ পাওয়ার অধিকারী কে? উত্তরে তিনি বললেন, তোমার মা। সে আবার জিজ্ঞেস করল,&lt;br&gt;&lt;br&gt;তারপর কে? তিনি বললেন, তোমার মা। সে পুনরায় জিজ্ঞেস করল, তারপর কে? তিনি বললেন, তোমার মা। সে আবার জিজ্ঞেস করল, তারপর কে? তিনি বললেন, তোমার পিতা' (ছহীহ বুখারী, হা/৫৯৭১; ছহীহ মুসলিম, হা/৬৬৬৪; মিশকাত, হা/৪৯১১)।&lt;br&gt;&lt;br&gt;
+এই হাদীছে প্রথমে তিনবার মায়ের কথা বলে চতুর্থবার পিতার কথা বলা হয়েছে। এতে বুঝা যায় যে, মায়ের মর্যাদা সবচেয়ে বেশি।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: قَالَ رَسُولُ اللهِ : رَغِمَ أَنْفُهُ ، رَغِمَ أَنْفُهُ، رَغِمَ أَنْفُهُ ، قِيلَ: مَنْ يَا رَسُولَ اللهِ؟ قَالَ: مَنْ أَدْرَكَ وَالِدَيْهِ عِنْدَ الْكِبَرِ، أَحَدَهُمَا أَوْ كِلَاهُمَا ثُمَّ لَمْ يَدْخُلِ الْجَنَّةَ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'তার নাক ধূলায় মলিন হোক (একথা তিনি তিন বার বললেন)। বলা হল, সে ব্যক্তি কে হে আল্লাহর রাসূল? তিনি বললেন, যে ব্যক্তি বৃদ্ধ পিতা-মাতাকে অথবা দুজনের একজনকে পেল অথচ (তাদের সেবা করে) সে জান্নাত লাভ করতে পারল না' (ছহীহ মুসলিম, হা/৬৬৭৫; মিশকাত, হা/৪৯১২)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ مُعَاوِيَةَ بْنِ جَاهِمَةَ جَاءَ إِلَى رَسُولِ اللهِ ﷺ فَقَالَ يَا رَسُولَ اللَّهِ أَرَدْتُ الْغَزْوَ وَجِئْتُكَ أَسْتَشِيرُكَ. فَقَالَ هَلْ لَكَ مِنْ أُمَّ». قَالَ نَعَمْ. فَقَالَ الْزَمْهَا فَإِنَّ الْجَنَّةَ عِنْدَ رِجْلِهَا».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+মু'আবিয়া ইবনু জাহিমা (রাঃ) হতে বর্ণিত, একদা আমার পিতা জাহিমা রাসূলুল্লাহ (ﷺ)-এর নিকট এসে বললেন, হে আল্লাহর রাসূল! আমি জিহাদে যেতে ইচ্ছুক। আমি আপনার নিকট পরামর্শ নিতে এসেছি। তখন তিনি জিজ্ঞাসা করলেন, তোমার মাতা আছেন কি? তিনি বললেন, হ্যাঁ। রাসূলুল্লাহ (ﷺ) বললেন, তুমি তাঁর সেবা কর। তাঁর পায়ের নিকট জান্নাত রয়েছে' (মুসনাদে আহমাদ, হা/১৫৯৩৭; নাসাঈ, হা/৩১০৪; মিশকাত, হা/৪৯৩৯)।&lt;br&gt;&lt;br&gt;
+অন্য বর্ণনায় এসেছে,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي أُمَامَةَ أَنَّ رَجُلًا قَالَ: يَا رَسُولَ اللهِ مَا حَقُّ الْوَالِدَيْنِ عَلَى وَلَدِهِمَا؟ قَالَ: «هُمَا جَنَّتُكَ وَنَارُكَ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ উমামা (রাঃ) হতে বর্ণিত, এক ব্যক্তি বললেন, হে আল্লাহর রাসূল ! সন্তানের উপর পিতামাতার কী হক্ক? তিনি বললেন, তারা উভয় তোমার জান্নাত ও জাহান্নাম' (ইবনু মাজাহ, হা/৩৬৬২; মিশকাত, হা/৪৯৪১)।&lt;br&gt;&lt;br&gt;
+উপরোক্ত হাদীছ দুটি দ্বারা বুঝা যায় যে, পিতামাতা সন্তানের জান্নাতে যাওয়ার মাধ্যম এবং জাহান্নাম থেকে পরিত্রাণ পাওয়ার উপায়। তাই তাদের&lt;br&gt;&lt;br&gt;সাথে সদাচরণ করে জান্নাত লাভের চেষ্টা করাই মুমিনের কর্তব্য। পিতামাতার নিকটে কোনো ছেলের স্ত্রী যদি অপছন্দনীয় হয়, তবে তাকে তালাক্ব দিতে হবে。&lt;br&gt;&lt;br&gt;
+এ মর্মে হাদীছে এসেছে,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي الدَّرْدَاءِ الله أَنَّ رَجُلًا أَتَاهُ، فَقَالَ: إِنَّ لِي امْرَأَةً وَإِنَّ أُمِّي تَأْمُرُنِي بِطَلَاقِهَا، فَقَالَ لَهُ أَبُو الدَّرْدَاءِ: سَمِعْتُ رَسُولَ اللهِ اللهِ يَقُولُ: الْوَالِدُ أَوْسَطُ أَبْوَابِ الْجَنَّةِ، فَإِنْ شِئْتَ فَحَافِظُ عَلَى الْبَابِ أَوْ ضَيِّع».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবু দারদা (রাঃ)-এর নিকট এক ব্যক্তি এসে বলল, আমার স্ত্রী আছে এবং আমার মাতা আমার স্ত্রীকে তালাক্ব দিতে বলছেন। আবু দারদা (রাঃ) তাকে বললেন, আমি রাসূলুল্লাহ (ﷺ)-কে বলতে শুনেছি, পিতা-মাতা হচ্ছেন জান্নাত লাভের উত্তম মাধ্যম। আপনি ইচ্ছা করলে তা হেফাযত করতে পারেন, নষ্টও করতে পারেন' (তিরমিযী, হা/১৯০০; মিশকাত, হা/৪৯২৮)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَسْمَاءَ بِنْتِ أَبِي بَكْرٍ قَالَتْ : قَدِمَتْ عَلَى أُمِّي وَهِيَ مُشْرِكَةً فِي عَهْدِ قُرَيْشٍ، فَقُلْتُ: يَا رَسُولَ اللهِ إِنَّ أُمِّي قَدِمَتْ عَلَيَّ وَهِيَ رَاغِبَةٌ، أَفَأَصِلُهَا؟ قَالَ: نَعَمْ صِلِيْهَا».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবুবকর-এর মেয়ে আসমা (রাঃ) হতে বর্ণিত, তিনি বলেন, আমার অমুসলিম মা, আমার নিকট আসতেন, আমি জিজ্ঞাসা করলাম, হে আল্লাহর রাসূল! আমার মা ইসলামের ব্যাপারে অনাগ্রহী, তিনি আমার নিকট আসেন, আমি তার সাথে কি সদ্ব্যবহার করব? তিনি বললেন, হ্যাঁ তার সাথে সদ্ব্যবহার কর' (ছহীহ বুখারী, হা/২৬২০; ছহীহ মুসলিম, হা/২৩৭২; মিশকাত, হা/৪৯১৩)।&lt;br&gt;&lt;br&gt;
+এই হাদীছ দ্বারা বুঝা যায় যে, পিতা মাতা অমুসলিম হলেও তাদের সাথে সদাচরণ করতে হবে। পিতামাতা নির্দেশ দিলে স্ত্রীকে তালাক দিতে হবে, যা উপরোক্ত হাদীছ দ্বারা প্রমাণিত হয়েছে।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ عَبْدِ اللَّهِ بْنِ عَمْرٍو قَالَ : قَالَ رَسُول الله ﷺ : «لَا يَدْخُلُ الْجَنَّةَ مَنَّانُ وَلَا عَاقُ وَلَا مُدْمِنُ خَمْرٍ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আব্দুল্লাহ ইবনু আমর (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, ইহসান করে খোঁটাদানকারী, মাতা-পিতার বিরুদ্ধাচরণকারী ও মদ্যপানকারী জান্নাতে প্রবেশ করবে না' (নাসাঈ, হা/৫৬৯০, সুনান আদ-দারেমী হা/২১৪৬; মিশকাত, হা/৪৯৩৩)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: قَالَ النَّبِيُّ  : السَّاعِي عَلَى الأَرْمَلَةِ وَالْمِسْكِينِ كَالسَّاعِي فِي سَبِيلِ اللهِ، وَأَحْسِبُهُ قَالَ كَالْقَائِمِ لَا يَفْتُرُ وَكَالصَّائِمِ النَّهَارَ لَا يُفْطِرُ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবু হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, নবী (ﷺ) বলেছেন, 'বিধবা ও মিসকীনের তত্ত্বাবধানকারী আল্লাহর রাস্তায় জিহাদকারীর মত। রাবী বলেন, আমার ধারণা, নবী এটাও বলেছেন, রাত্রি জাগরণ করে ইবাদতকারীর মত, যে অলসতা করে না এবং ঐ ছিয়াম পালনকারীর মত, যে কখনও ছিয়াম ভঙ্গ করে না' (ছহীহ বুখারী, হা/৬০০৭; ছহীহ মুসলিম, হা/৭৬৫৯; মিশকাত হা/৪৯৫১)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ عَبْدِ اللَّهِ بْنِ عَمْرِو بْنِ الْعَاصِ عَنِ النَّبِيِّ ﷺ قَالَ : الْكَبَائِرُ الْإِشْرَاكُ بِاللَّهِ وَعُقُوْقُ الْوَالِدَيْنِ وَقَتْلُ النَّفْسِ وَالْيَمِينُ الْغَمُوسُ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আব্দুল্লাহ ইবনু আমর ইবনুল আছ (রাঃ) হতে বর্ণিত, নবী (ﷺ) বলেছেন, বড় গুনাহ হচ্ছে আল্লাহর সাথে শরীক করা, পিতামাতার অবাধ্য হওয়া, মানুষকে হত্যা করা এবং মিথ্যা কসম করা' (আত-তারগীব, হা/৩৫৬৮)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنِ ابْنِ عُمَرَ عَنْ رَسُولِ اللهِ ﷺ قَالَ : ثَلَاثَةٌ لَا يَنْظُرُ اللَّهُ إِلَيْهِمْ يَوْمَ الْقِيَامَةِ الْعَاقُ لِوَالِدَيْهِ وَمُدْمِنُ الْخَمْرِ وَالْمَنَّانُ عَطَاءَهُ وَثَلَاثَةُ لَا يَدْخُلُوْنَ الْجَنَّةَ الْعَاقُ لِوَالِدَيْهِ وَالدَّيَوْتُ وَالرَجْلَةُ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+ইবনু উমার (রাঃ) হতে বর্ণিত, রাসূলুল্লাহ (ﷺ) বলেছেন, 'কিয়ামতের দিন আল্লাহ তিন শ্রেণীর মানুষের প্রতি দয়ার দৃষ্টি দিবেন না। (১) পিতামাতার অবাধ্য ব্যক্তি (২) নিয়মিত নেশাদার দ্রব্য পানকারী (৩) দান করার পর খোটা দানকারী। তিনি আবার বলেন, তিন শ্রেণীর মানুষ জান্নাতে যাবে না। (১) পিতামাতার অবাধ্য ব্যক্তি, (২) দায়ূছ ব্যক্তি (৩) পুরুষের বেশধারী নারী' (আত- তারগীব, হা/২৫১১)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;وَعَنْ أَبِي أُمَامَةَ ، قَالَ : قَالَ رَسُوْلُ اللهِ ﷺ : ثَلَاثَةٌ لَا يَقْبَلُ اللَّهُ عَزَّ وَجَلَّ مِنْهُمْ صَرْفًا وَلَا عَدْلًا عَاقٌ وَ مَنَّانُ وَمُكَذِّبُ بِقَدَرٍ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ উমামা (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'তিন শ্রেণীর মানুষ রয়েছে, যাদের ফরয ও নফল ইবাদত আল্লাহ কবুল করবেন না। (১) পিতামাতার অবাধ্য ব্যক্তি, (২) খোটা দানকারী এবং (৩) ভাগ্যকে অস্বীকারকারী' (আত-তারগীব, হা/৩৫৭৩)।&lt;br&gt;&lt;br&gt;আবু হুরায়রা (রাঃ) বলেন, রাসূল (ﷺ) বলেছেন, 'পিতামাতার অনুগত হলে বয়স বৃদ্ধি পায়। মিথ্যা কথা রুযী কমিয়ে দেয়। দু'আ নির্ধারিত ভাগ্যের পরিবর্তন ঘটায়' (আত-তারগীব, হা/৪২০৩)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنِ ابْنِ عَبَّاسٍ قَالَ لَمَّا كَانَ بَيْنَ إِبْرَاهِيمَ وَبَيْنَ أَهْلِهِ مَا كَانَ، خَرَجَ بِإِسْمَاعِيلَ وَأَمْ إِسْمَاعِيلَ، وَمَعَهُمْ شَنَّةٌ فِيهَا مَاءُ ، فَجَعَلَتْ أُمُّ إِسْمَاعِيلَ تَشْرَبُ مِنَ السُّنَّةِ فَيَدِرُّ لَبَنُهَا عَلَى صَبِيِّهَا حَتَّى قَدِمَ مَكَّةَ، فَوَضَعَهَا تَحْتَ دَوْحَةٍ ، ثُمَّ رَجَعَ إِبْرَاهِيمُ إِلَى أَهْلِهِ، فَاتَّبَعَتْهُ أُمُّ إِسْمَاعِيلَ، حَتَّى لَمَّا بَلَغُوا كَدَاءً نَادَتْهُ مِنْ وَرَائِهِ يَا إِبْرَاهِيمُ إِلَى مَنْ تَتْرُكُنَا قَالَ إِلَى اللهِ . قَالَتْ رَضِيتُ بِاللهِ . قَالَ فَرَجَعَتْ فَجَعَلَتْ تَشْرَبُ مِنَ الشَّنَّةِ وَيَدِرُّ لَبَنُهَا عَلَى صَبِيِّهَا، حَتَّى لَمَّا فَنِيَ الْمَاءُ قَالَتْ لَوْ ذَهَبْتُ فَنَظَرْتُ لَعَلَّى أُحِسُّ أَحَدًا . قَالَ فَذَهَبَتْ فَصَعِدَتِ الصَّفَا فَنَظَرَتْ وَنَظَرَتْ هَلْ تُحِسُّ أَحَدًا فَلَمْ تُحِسَّ أَحَدًا، فَلَمَّا بَلَغَتِ الْوَادِيَ سَعَتْ وَأَتَتِ الْمَرْوَةَ فَفَعَلَتْ ذَلِكَ أَشْوَاطًا، ثُمَّ قَالَتْ لَوْ ذَهَبْتُ فَنَظَرْتُ مَا فَعَلَ - تَعْنِي الصَّبِيَّ - فَذَهَبَتْ فَنَظَرَتْ، فَإِذَا هُوَ عَلَى حَالِهِ كَأَنَّهُ يَنْشَعُ لِلْمَوْتِ، فَلَمْ تُقِرَّهَا نَفْسُهَا، فَقَالَتْ لَوْ ذَهَبْتُ فَنَظَرْتُ لَعَلَّى أُحِسُّ أَحَدًا، فَذَهَبَتْ فَصَعِدَتِ الصَّفَا فَنَظَرَتْ وَنَظَرَتْ فَلَمْ تُحِسَّ أَحَدًا، حَتَّى أَتَمَّتْ سَبْعًا، ثُمَّ قَالَتْ لَوْ ذَهَبْتُ فَنَظَرْتُ مَا فَعَلَ، فَإِذَا هِيَ بِصَوْتٍ فَقَالَتْ أَغِتْ إِنْ كَانَ عِنْدَكَ خَيْرُ . فَإِذَا جِبْرِيلُ، قَالَ فَقَالَ بِعَقِبِهِ هَكَذَا ، وَغَمَزَ عَقِبَهُ عَلَى الأَرْضِ ، قَالَ فَانْبَثَقَ الْمَاءُ، فَدَهَشَتْ أُمُّ إِسْمَاعِيلَ فَجَعَلَتْ تَحْفِرُ . قَالَ فَقَالَ أَبُو الْقَاسِمِ اللهِ لَوْ تَرَكَتْهُ كَانَ الْمَاءُ ظَاهِرًا». قَالَ فَجَعَلَتْ تَشْرَبُ مِنَ الْمَاءِ، وَيَدِرُّ لَبَنُهَا عَلَى صَبِيّهَا - قَالَ - فَمَرَّ نَاسٌ مِنْ جُرْهُم بِبَطْنِ الْوَادِي، فَإِذَا هُمْ بِطَيْرٍ، كَأَنَّهُمْ أَنْكَرُوا ذَاكَ، وَقَالُوا مَا يَكُونُ الطَّيْرُ إِلا عَلَى مَاءٍ . فَبَعَثُوا رَسُولَهُمْ، فَنَظَرَ فَإِذَا هُمْ بِالْمَاءِ، فَأَتَاهُمْ فَأَخْبَرَهُمْ فَأَتَوْا إِلَيْهَا، فَقَالُوا يَا أُمَّ إِسْمَاعِيلَ، أَتَأْذَنِينَ لَنَا أَنْ نَكُونَ مَعَكِ أَوْ نَسْكُنَ مَعَكِ فَبَلَغَ ابْنُهَا فَنَكَحَ فِيهِمُ امْرَأَةً ، قَالَ ثُمَّ إِنَّهُ بَدَا لِإِبْرَاهِيمَ فَقَالَ لَأَهْلِهِ إِنِّي مُطَّلِعُ تَرِكَتِي . قَالَ فَجَاءَ فَسَلَّمَ فَقَالَ أَيْنَ إِسْمَاعِيلُ فَقَالَتِ امْرَأَتُهُ ذَهَبَ يَصِيدُ . قَالَ قُولِي لَهُ إِذَا جَاءَ غَيِّرْ عَتَبَةَ بَابِكَ . فَلَمَّا جَاءَ أَخْبَرَتْهُ قَالَ أَنْتِ ذَاكِ فَاذْهَبِي إِلَى أَهْلِكِ . قَالَ ثُمَّ إِنَّهُ بَدَا لِإِبْرَاهِيمَ فَقَالَ لِأَهْلِهِ إِنِّى مُطَّلِعُ تَرِكَتِي . قَالَ فَجَاءَ فَقَالَ أَيْنَ إِسْمَاعِيلُ فَقَالَتِ امْرَأَتُهُ ذَهَبَ يَصِيدُ، فَقَالَتْ أَلَا تَنْزِلُ فَتَطْعَمَ وَتَشْرَبَ فَقَالَ وَمَا طَعَامُكُمْ وَمَا شَرَابُكُمْ قَالَتْ طَعَامُنَا اللَّحْمُ، وَشَرَابُنَا الْمَاءُ . قَالَ اللهُمَّ بَارِكْ لَهُمْ فِي طَعَامِهِمْ وَشَرَابِهِمْ . قَالَ فَقَالَ أَبُو الْقَاسِمِ ﷺ بَرَكَةُ بِدَعْوَةِ إِبْرَاهِيمَ. قَالَ ثُمَّ إِنَّهُ بَدَا الإِبْرَاهِيمَ فَقَالَ لِأَهْلِهِ إِنِّي مُطَّلِعُ تَرِكَتِي . فَجَاءَ فَوَافَقَ إِسْمَاعِيلَ مِنْ وَرَاءِ زَمْزَمَ، يُصْلِحُ نَبْلاً لَهُ، فَقَالَ يَا إِسْمَاعِيلُ، إِنَّ رَبَّكَ أَمَرَنِي أَنْ أَبْنِيَ لَهُ بَيْتًا . قَالَ أَطِعْ رَبَّكَ . قَالَ إِنَّهُ قَدْ أَمَرَنِي أَنْ تُعِينَنِي عَلَيْهِ . قَالَ إِذَا أَفْعَلَ ، أَوْ كَمَا قَالَ . قَالَ فَقَامَا فَجَعَلَ إِبْرَاهِيمُ يَبْنِي، وَإِسْمَاعِيلُ يُنَاوِلُهُ الْحِجَارَةَ، وَيَقُولَانِ رَبَّنَا تَقَبَّلْ مِنَّا إِنَّكَ أَنْتَ السَّمِيعُ الْعَلِيمُ) قَالَ حَتَّى ارْتَفَعَ الْبِنَاءُ وَضَعُفَ الشَّيْخُ عَلَى نَقْلِ الْحِجَارَةِ، فَقَامَ عَلَى حَجَرِ الْمَقَامِ، فَجَعَلَ يُنَاوِلُهُ الْحِجَارَةَ، وَيَقُولَانِ رَبَّنَا تَقَبَّلْ مِنَّا إِنَّكَ أَنْتَ السَّمِيعُ الْعَلِيمُ .&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+ইবনু আব্বাস (রাঃ) হতে বর্ণিত, তিনি বলেন, যখন ইবরাহীম (আঃ) ও তাঁর স্ত্রী (সারার) মাঝে যা হবার হয়ে গেল। তখন ইবরাহীম আপাইরিস সালাম শিশুপুত্র ইসমাঈল এবং তার মাকে নিয়ে বের হলেন। তাদের সঙ্গে একটি থলে ছিল, যাতে পানি ছিল। ইসমাঈল (আঃ)-এর মা মশক হতে পানি পান করতেন। ফলে শিশুর জন্য তার স্তনে দুধ বাড়তে থাকত। অবশেষে ইবরাহীম (আঃ) মক্কায় পৌঁছে হাজেরাকে একটি বিরাট গাছের নিচে থাকার ব্যবস্থা করে দিলেন। অতঃপর ইবরাহীম (আঃ) স্বীয় পরিবারের (সারার) নিকট ফিরে চললেন। তখন ইসমাঈল (আঃ)-এর মা কিছু দূর পর্যন্ত তার অনুসরণ করলেন। অবশেষে যখন 'কাদা' নামক স্থানে পৌঁছলেন, তখন তিনি পিছন হতে ডেকে বললেন, হে ইবরাহীম! আপনি আমাদেরকে কার নিকট রেখে যাচ্ছেন? ইবরাহীম (আঃ) বললেন, আল্লাহর কাছে। হাজেরা (আঃ) বললেন, আমি আল্লাহর প্রতি সন্তুষ্ট। রাবী বলেন, অতঃপর হাজেরা (আঃ) ফিরে আসলেন এবং, তিনি মশক হতে পানি পান করলেন। আর শিশুর জন্য দুধ বাড়লো। অবশেষে যখন পানি শেষ হয়ে গেল। তখন ইসমাঈল আলাইহি-এর মা বললেন, আমি যদি গিয়ে এদিকে সেদিকে তাকাতাম, তাহলে হয়তো কোনো মানুষ দেখতে পেতাম। রাবী বলেন, অতঃপর হাজেরা (আঃ) গেলেন এবং ছাফা পাহাড়ে উঠলেন। আর এদিকে ওদিকে তাকালেন এবং কাউকে দেখেন কিনা এজন্য বিশেষভাবে তাকিয়ে দেখলেন। কিন্তু কাউকেও দেখতে পেলেন না। তখন দ্রুত বেগে মারওয়া পাহাড়ে এসে গেলেন এবং এভাবে কয়েক চক্কর দিলেন। পুনরায় তিনি বললেন, যদি গিয়ে দেখতাম যে, শিশুটি কী করছে? অতঃপর তিনি গেলেন এবং দেখতে পেলেন যে, সে তার অবস্থায়ই আছে। সে যেন মরণাপন্ন হয়ে গেছে। এতে তার মন স্বস্তি পাচ্ছিল না। তখন তিনি বললেন, যদি সেখানে যেতাম এবং এদিকে সেদিকে তাকিয়ে দেখতাম, সম্ভবত কাউকে দেখতে পেতাম। অতঃপর তিনি গেলেন এবং, ছাফা পাহাড়ের উপর উঠলেন এবং এদিক সেদিক দেখলেন এবং গভীরভাবে তাকিয়ে দেখলেন। কিন্তু কাউকে দেখতে পেলেন না। এভাবে তিনি সাতটি&lt;br&gt;&lt;br&gt;সালাম চক্কর পূর্ণ করলেন। তখন তিনি বললেন, যদি যেতাম তাহলে দেখতাম, সে (শিশুটি) কী করছে? হঠাৎ তিনি একটি শব্দ শুনতে পেলেন। অতঃপর তিনি মনে মনে বললেন, যদি আপনার কোনো সাহায্য করার থাকে, তবে আমাকে সাহায্য করুন। হঠাৎ তিনি জিবরাঈল (আঃ)-কে দেখতে পেলেন। রাবী বলেন, তখন তিনি (জিবরাঈল) তার পায়ের গোড়ালী দ্বারা এরূপ করলেন। হঠাৎ গোড়ালি দ্বারা জমিনের উপর আঘাত করলেন। রাবী বলেন, তখনি পানি বেরিয়ে আসল। এ দেখে ইসমাঈল আলাইহি-এর মা অস্থির হয়ে গেলেন এবং গর্ত খুঁড়তে লাগলেন। রাবী বলেন, এ প্রসঙ্গে আবুল কাসেম (রাসূলুল্লাহ (ﷺ)) বলেছেন, হাজেরা (আঃ) যদি একে তার অবস্থার উপর ছেড়ে দিতেন, তাহলে পানি বিস্তৃত হয়ে যেত। রাবী বলেন, তখন হাজেরা (আঃ) পানি পান করতে লাগলেন এবং তার সন্তানের জন্য তার দুধ বাড়তে থাকে। রাবী বলেন, অতঃপর জুরহুম গোত্রের এক দল লোক উপত্যকার নিচু ভূমি দিয়ে অতিক্রম করছিল। হঠাৎ তারা দেখল কিছু পাখি উড়ছে। তারা যেন তা বিশ্বাসই করতে পারছিল না। আর তারা বলতে লাগল, এসব পাখিতো পানি ব্যতীত কোথাও থাকতে পারে না। তখন তারা সেখানে তাদের একজন পাঠাল। সেখানে গিয়ে দেখল, সেখানে পানি আছে। তখন সে তার দলের লোকদের নিকট ফিরে আসল এবং তাদেরকে সংবাদ দিল। অতঃপর তারা হাজেরা (আঃ)-এর নিকট এসে বললো, হে ইসমাঈলের মা! আপনি কি আমাদেরকে আপনার নিকট থাকা অথবা (রাবী সন্দেহ)) আপনার নিকট বসবাস করার অনুমতি দিবেন?অতঃপর তার ছেলে বয়ঃপ্রাপ্ত হল। তখন তিনি (ইসমাঈল) জুরহুম গোত্রেরই একটি মেয়েকে বিয়ে করলেন। রাবী বলেন, পুনরায় ইবরাহীম (আঃ)-এর মনে জাগল, তখন তিনি তার স্ত্রী (সারাকে) বললেন, আমি আমার পরিত্যক্ত পরিজনের খবর নিতে চাই। রাবী বলেন, অতঃপর তিনি আসলেন এবং সালাম দিলেন। তিনি জিজ্ঞাসা করলেন, ইসমাঈল কোথায়? ইসমাঈল (আঃ)-এর স্ত্রী বললেন, তিনি শিকারে গেছেন। তিনি পুত্রবধূকে তাদের অবস্থা সম্পর্কে জিজ্ঞাসা করলেন। সে বলল, আমরা অতি দুরাবস্থায়, অতি টানাটানি ও খুব কষ্টে আছি। ইবরাহীম বললেন, সে যখন আসবে তখন তুমি তাকে আমার এ নির্দেশের কথা বলবে, তুমি তোমার ঘরের চৌকাঠ খানা বদলিয়ে ফেলো। ইসমাঈল (আঃ) যখন আসলেন, তখন স্ত্রী তাকে খবরটি জানালেন। তিনি স্ত্রীকে বললেন, তুমিই সেই চৌকাঠ। অতএব তুমি তোমার পরিবারের নিকট চলে যাও। রাবী বলেন, অতঃপর ইবরাহীম আলাইরি-এর আবার মনে পড়লো। তখন তিনি স্ত্রীকে (সারা) বললেন, আমি আমার নির্বাসিত পরিবারের খবর নিতে সালাম&lt;br&gt;&lt;br&gt;সালাম চাই। রাবী বলেন, অতঃপর তিনি সেখানে আসলেন এবং জিজ্ঞাসা করলেন, ইসমাঈল কোথায়? ইসমাঈল (আঃ)-এর স্ত্রী বললেন, তিনি শিকারে গেছেন। পুত্রবধূ তাকে বললেন, আপনি কি আমাদের এখানে অবস্থান করবেন না? কিছু পানাহার করবেন না? তখন ইবরাহীম (আঃ) বললেন, তোমাদের খাদ্য ও পানীয় কী? পুত্রবধূ বলল, আমাদের খাদ্য হল গোশত এবং পানীয় হল পানি। তখন ইবরাহীম (আঃ) দু'আ করলেন, হে আল্লাহ! তাদের খাদ্য এবং পানীয় দ্রব্যের মধ্যে বরকত দিন। রাবী বলেন, আবুল কাসেম বলেছেন, ইবরাহীম (আঃ)-এর দু'আর কারণেই বরকত রয়েছে। রাবী বলেন, আবার কিছু দিন পর ইবরাহীম (আঃ)-এর মনে তাঁর নির্বাসিত পরিজনের কথা জাগল। তখন তিনি তাঁর স্ত্রীকে (সারা) বললেন, আমি আমার পরিত্যক্ত পরিজনের খবর নিতে চাই। অতঃপর তিনি এলেন এবং ইসমাঈলের দেখা পেলেন, যে সময়, তিনি যমযম কূপের পিছনে বসে তার একটি তীর মেরামত করছেন। তখন ইবরাহীম (আঃ) ডেকে বললেন, হে ইসমাঈল! তোমার রব তাঁর জন্য এক খানা ঘর নির্মাণ করতে আমাকে নির্দেশ দিয়েছেন। ইসমাঈল (আঃ) বললেন, আপনার রবের নির্দেশ পালন করুন। ইবরাহীম (আঃ) বললেন, তিনি আমাকে এও নির্দেশ দিয়েছেন যে, তুমি যেন আমাকে এ বিষয়ে সহায়তা কর। ইসমাঈল (আঃ) বললেন, তাহলে আমি তা করব অথবা তিনি অনুরূপ কিছু বলেছিলেন। রাবী বলেন, অতঃপর উভয়ে উঠে দাঁড়ালেন। ইবরাহীম (আঃ) ইমারত বানাতে লাগলেন। আর ইসমাঈল (আঃ) তাঁকে পাথর এনে দিতে লাগলেন। আর তারা উভয়ে সালাম দু'আ করছিলেন, হে আমাদের রব! আপনি আমাদের এ কাজ কবুল করুন। আপনি তো সবকিছু শোনেন এবং জানেন। রাবী বলেন, এরই মধ্যে প্রাচীর উঁচু হয়ে গেল আর বৃদ্ধ ইবরাহীম (আঃ) এতটা উঠতে দুর্বল হয়ে পড়লেন। তখন তিনি (মাকামে ইবরাহীমের) পাথরের উপর দাঁড়ালেন। ইসমাঈল তাঁকে পাথর এগিয়ে দিতে লাগলেন। আর উভয়ে এ দু'আ পড়তে লাগলেন, হে আমাদের রব! আপনি আমাদের এ কাজটুকু কবুল করুন। নিঃসন্দেহে আপনি সবকিছু শোনেন ও জানেন (বাক্বারা, ১২৭; ছহীহ বুখারী, হা/৩৩৬৫)।&lt;br&gt;&lt;br&gt;&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>স্ত্রীর সাথে সদাচরণকারী</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>স্ত্রীর সাথে সদাচরণকারী</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>&lt;div class="page-text"&gt;&lt;br&gt;আদর্শ পুরুষ হিসাবে গণ্য হওয়ার জন্য মানুষের মধ্যে আল্লাহর ইবাদত- বন্দেগী ছাড়াও যেসব গুণাবলী থাকা অতীব জরুরী তন্মধ্যে অন্যতম হচ্ছে পিতামাতা, আত্মীয়-স্বজন, প্রতিবেশী ও স্ত্রীর সাথে সদাচরণ করা। কেননা স্ত্রী হচ্ছে জীবনের সার্বক্ষণিক সঙ্গী। তার সাথে সদ্ব্যবহার না করলে দাম্পত্য জীবনে নানা সমস্যা সৃষ্টি হয়। পরিবার পরিণত হয় অশান্তির আকারে। তাই তার সাথে উত্তম আচরণ করা আবশ্যক। আল্লাহ বলেন,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;وَعَاشِرُوهُنَّ بِالْمَعْرُوْفِ )&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+'তোমরা তাদের (স্ত্রীদের) সাথে সৎভাবে জীবন যাপন করো' (নিসা, ১৯)।&lt;br&gt;&lt;br&gt;
+এই আয়াত দ্বারা প্রতীয়মান হয় যে, স্ত্রীদের সাথে ভালো ব্যবহার করতে হবে。&lt;br&gt;&lt;br&gt;
+স্ত্রী যাতে স্বামীর অবাধ্য না হয় সে জন্য বিবাহের সময় সতী-সাধ্বী, বংশীয়া ও ধার্মিক মেয়ে দেখে বিবাহ করা উচিত। কেননা রাসূলুল্লাহ (ﷺ) বলেছেন, সমস্ত দুনিয়াই সম্পদ। আর দুনিয়ার শ্রেষ্ঠ সম্পদ হচ্ছে সতী-সাধ্বী নারী' (ছহীহ মুসলিম, হা/৩৭১৬; নাসাঈ, হা/৩২৩২; মিশকাত, হা/৩০৮৩)।&lt;br&gt;&lt;br&gt;
+অন্য হাদীছে রাসূলুল্লাহ (ﷺ) বিবাহের ক্ষেত্রে নারীদের দ্বীনদারিতাকেই প্রাধান্য দিতে বলেছেন (ছহীহ বুখারী, হা/৫০৯০; ছহীহ মুসলিম, হা/৩৭০৮; আবূ দাউদ, হা/২০৪৭)।&lt;br&gt;&lt;br&gt;
+স্ত্রীদের সাথে ব্যবহার সম্পর্কে হাদীছে এসেছে,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: قَالَ رَسُولُ اللهِ : اسْتَوْصُوا بِالنِّسَاءِ خَيْرًا فَإِنَّهُنَّ خُلِقْنَ مِنْ ضِلَعٍ وَإِنَّ أَعْوَجَ شَيْءٍ فِي الضَّلَعِ أَعْلَاهُ فَإِنْ ذَهَبْتَ تُقِيمُهُ كَسْرَتَهُ، وَإِنْ تَرَكْتَهُ لَمْ يَزَلْ أَعْوَجَ فَاسْتَوْصُوا بِالنِّسَاءِ»&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, তোমরা, স্ত্রীদের কল্যাণ সাধনের জন্য উপদেশ দিতে থাক। কেননা তারা&lt;br&gt;&lt;br&gt;পাঁজরের বাঁকা হাড় হতে সৃষ্টি। পাঁজরের উপরের হাড় হয় সর্বাপেক্ষা বাঁকা। যদি তুমি সোজা করতে যাও, তবে তা ভেঙ্গে যাবে। আর যদি ঐভাবে রেখে দাও, তাহলে বাঁকাই থেকে যাবে। অতএব তোমরা নারীদের সাথে চলার জন্য সদ্ব্যবহারের উপদেশ গ্রহণ করো' (ছহীহ বুখারী, হা/৩৩৩১; ছহীহ মুসলিম, হা/৩৭২০; মিশকাত, হা/৩২৩৮)।&lt;br&gt;&lt;br&gt;
+জোর করে সংশোধনের চেষ্টা করা উচিত নয়। তার দুর্বল দিক দেখেও না দেখার মত ভাব দেখিয়ে উপদেশ দিতে হবে। গুনাহ না হলে তার চাহিদা মত চলার চেষ্টা করতে হবে। নম্র আচরণের মাধ্যমে তার মন জয় করার চেষ্টা করতে হবে। আর এভাবে তাকে সঠিক পথে চালানোর চেষ্টা অব্যাহত রাখতে হবে।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ عَبْدِ اللَّهِ بْنِ زَمْعَةَ عَنِ النَّبِيِّ ﷺ قَالَ لا يَجْلِدُ أَحَدُكُمُ امْرَأَتَهُ جَلْدَ الْعَبْدِ، ثُمَّ يُجَامِعُهَا فِي آخِرِ الْيَوْمِ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আব্দুল্লাহ ইবনু যাম'আ (রাঃ) হতে বর্ণিত, নবী (ﷺ) বলেছেন, 'তোমাদের কেউ যেন ক্রীতদাসকে চাবুক মারার ন্যায় নিজের স্ত্রীকে লাঠিপেটা না করে এবং দিন শেষে তার সাথে সহবাস করে (ছহীহ বুখারী, হা/৫২০৪; ছহীহ ইবনু হিব্বান হা/৪১৯০; মিশকাত, হা/৩২৪২)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ حَكِيمِ بْنِ مُعَاوِيَةَ الْقُشَيْرِي عَنْ أَبِيهِ قَالَ: قُلْتُ: يَا رَسُولَ اللَّهِ مَا حَقٌّ زَوْجَةِ أَحَدِنَا عَلَيْهِ؟ قَالَ: أَنْ تُطْعِمَهَا إِذَا طَعِمْتَ وَتَكْسُوَهَا إِذَا اكْتَسَيْتَ وَلَا تَضْرِبِ الْوَجْهَ وَلَا تُقَبِّحْ وَلَا تَهْجُرْ إِلَّا فِي الْبَيْتِ»&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+হাকীম ইবনু মু'আবিয়া আল-কুশায়রী (রাঃ) তার পিতা হতে বর্ণনা করেন, তার পিতা বলেছেন, আমি রাসূলুল্লাহ (ﷺ)-কে বললাম, হে আল্লাহর রাসূল! আমাদের উপর স্ত্রীর হক্ক কী? তিনি বললেন, তুমি যখন খাবে, তখন তোমার স্ত্রীকে খাওয়াবে। যখন তুমি পোশাক পরবে, তখন তাকেও পরাবে। তার মুখে মারবে না। তাকে অশ্লীল ভাষায় গালি দিবে না। বাড়িতে ব্যতীত তাকে ছাড়বে না' (আবূ দাউদ, হা/২১৪৪; মুসনাদে আহমাদ, হা/২০৫৫৭; মিশকাত হা/৩২৫৯)।&lt;br&gt;&lt;br&gt;
+☑ এই হাদীছে পাঁচটি বিষয়ে স্ত্রীর প্রতি লক্ষ্য রাখতে বলা হয়েছে- (১) স্বামীর সামর্থ্য অনুযায়ী খাওয়া-দাওয়ার ব্যবস্থা করতে হবে। এ ব্যাপারে নিজের বিষয়টিকে প্রাধান্য দেওয়া যাবে না। কোনোক্রমেই তাদের সাথে কৃপণতা করা যাবে না。&lt;br&gt;&lt;br&gt;(২) পরিধানের পোশাক-পরিচ্ছদের ব্যাপারে খেয়াল রাখতে হবে। সাজসজ্জা নারীদের পছন্দনীয়। তাই তাদের জন্য স্বামী তার সাধ্যমত প্রসাধনী ও সাজসজ্জার জিনিস সংগ্রহ করে দিবে। কেননা তারা সাজসজ্জার মাধ্যমে স্বামীকে আকৃষ্ট করতে সচেষ্ট হয়। (৩) মুখে মারা নিষেধ। (৪) স্ত্রীদের সাথে সর্বদা সদয় হয়ে চলতে হবে। তাদের সাথে নির্দয় আচরণ হতে বিরত থাকতে হবে। তাদের সাথে কঠোরতা পরিহার করতে হবে। তাদেরকে অকথ্য ভাষায় গালিগালাজ করা, অতিরিক্ত মারধর করা, তাদের কাজকর্মের দোষ-ত্রুটি খুঁজে বেড়ানো যাবে না। (৫) জরুরী প্রয়োজন ছাড়া বাড়ির বাইরে যেতে দেওয়া যাবে না। জরুরী দুর্ঘটনা ছাড়া হাটে, বাজারে, বিয়ের বাড়িতে যেতে দেওয়া যাবে না。&lt;br&gt;&lt;br&gt;
+মোদ্দাকথা, তাদের সাথে ভালোবাসার সাথে আচরণ করতে হবে। এখানে উপরোক্ত বিষয়গুলোর প্রতি খেয়াল রাখতে হবে। তবে সতর্ক করার জন্য হালকা প্রহার করা যায়। আল্লাহ বলেন,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;وَاللَّاتِي تَخَافُونَ نُشُوزَهُنَّ فَعِظُوهُنَّ وَاهْجُرُوهُنَّ فِي الْمَضَاجِعِ وَاضْرِبُوهُنَّ )&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+'তোমরা তাদের নাফরমানীর আশংকা করলে তাদের হালকা প্রহার করো' (নিসা, ৩৪)।&lt;br&gt;&lt;br&gt;
+রাসূলুল্লাহ (ﷺ) বলেন,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;وَلَا تَرْفَعْ عَنْهُمْ عَصَاكَ أَدَبًا»&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+'তোমরা পরিবারের উপর হতে শিষ্টাচারের লাঠি উঠিয়ে নিয়ো না' (মুসনাদে আহমাদ, হা/২২৭২৬; মিশকাত, হা/৬১)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: قَالَ رَسُولُ اللهِ ﷺ : «إِذَا قَاتَلَ أَحَدُكُمْ فَلْيَجْتَنِبِ الْوَجْهَ، فَإِنَّ اللَّهَ خَلَقَ آدَمَ عَلَى صُورَتِهِ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'যখন তোমাদের কোনো ব্যক্তি কাউকে মারবে সে যেন মুখের উপর না মারে। কেননা, আল্লাহ আদমকে তার আকৃতিতে সৃষ্টি করেছেন' (ছহীহ মুসলিম, হা/৬৮২১; মুসনাদে আহমাদ, হা/১০২২২; মিশকাত, হা/৩৫২৫)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ جَابِرِ بْنِ عَبْدِ اللهِ الله عَنِ النَّبِيِّ ﷺ فِي حَدِيْثِ الْحَجِّ بِطُوْلِهِ قَالَ فِي ذِكْرِ النِّسَاءِ: «وَلَهُنَّ عَلَيْكُمْ رِزْقُهُنَّ وَكِسْوَتُهُنَّ بِالْمَعْرُوفِ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;জাবের ইবনু আব্দুল্লাহ (রাঃ) হতে বর্ণিত, নবী (ﷺ) হজ্জের লম্বা হাদীছ বলতে গিয়ে মহিলাদের সম্পর্কে বলেন, 'তোমরা তাদের জন্য সুন্দর রুযীর ব্যবস্থা করবে এবং সুন্দর পরিধানের ব্যবস্থা করবে' (ছহীহ মুসলিম, হা/৩০০৯; আবু দাউদ, হা/১৯০৭; মিশকাত, হা/২৫৫৫)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ عَائِشَةَ قَالَتْ كَانَ الْخَبَشُ يَلْعَبُونَ بِحِرَابِهِمْ، فَسَتَرَنِي رَسُولُ اللَّهِ ﷺ وَأَنَا أَنْظُرُ، فَمَا زِلْتُ أَنْظُرُ حَتَّى كُنْتُ أَنَا أَنْصَرِفُ فَاقْدُرُوا قَدْرَ الْجَارِيَةِ الحَدِيثَةِ السِّنِّ تَسْمَعُ اللَّهْوَ .&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আয়েশা (রাঃ) হতে বর্ণিত, তিনি বলেন, একদা হাবশীরা তাদের বর্শা নিয়ে খেলা করছিল। তখন রাসূলুল্লাহ (ﷺ) আমাকে নিয়ে পর্দা করে তাঁর পিছনে দাঁড় করিয়ে দিলেন এবং আমি সেই খেলা দেখছিলাম যতক্ষণ আমার ভালো লাগছিল। যতক্ষণ স্বেচ্ছায় আমি সেই স্থান ত্যাগ না করতাম। সুতরাং তোমরা অনুমান করতে পার কম বয়সের মেয়েরা আমোদ-প্রমোদ, খেল- তামাশা দেখতে ভালোবাসে' (ছহীহ বুখারী, হা/৫১৯০; নাসাঈ, হা/১৫৯৪)।&lt;br&gt;&lt;br&gt;
+রাসূলুল্লাহ (ﷺ) স্বীয় স্ত্রীদের প্রতি কতটা সদয় ছিলেন এই হাদীছ তার উজ্জ্বল প্রমাণ। প্রত্যেক মুসলিম পুরুষকে অনুরূপ স্ত্রীর প্রতি সদয় হতে হবে。&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: مَا عَابَ النَّبِيُّ اللهِ طَعَامًا قَطُّ إِنْ اشْتَهَاهُ أَكَلَهُ وَإِنْ كَرِهَهُ تَرَكَهُ.&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, নবী (ﷺ) কখনও খাবারের দোষ-ত্রুটি বর্ণনা করেননি। তাঁর ভালো লাগলে তিনি খেতেন, ভালো না লাগলে রেখে দিতেন (ছহীহ বুখারী, হা/৩৫৬৩; আবু দাউদ, হা/৩৭৬৩; মুসনাদে আহমাদ, হা/১০২৪৭)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ سَعْدِ بْنِ أَبِي وَقَّاصٍ قَالَ: إِنَّ رَسُولَ اللهِ ﷺ قَالَ : وَإِنَّكَ لَنْ تُنْفِقَ نَفَقَةً تَبْتَغِي بِهَا وَجْهَ اللَّهِ إِلَّا أُجِرْتَ بِهَا، حَتَّى مَا تَجْعَلُ فِي فِي امْرَأَتِكَ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+সা'দ ইবনু আবী ওয়াক্কাছ (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'তুমি আল্লাহর সন্তুষ্টির জন্য যেকোনো ব্যয়ই কর না কেন, এর বিনিময় তোমাকে ছাওয়াব দেওয়া হবে। এমনকি তুমি তোমার স্ত্রীর মুখে যে খাদ্য তুলে দাও তার বিনিময়েও ছওয়াব দেওয়া হবে' (ছহীহ বুখারী, হা/১২৯৫; ছহীহ মুসলিম, হা/৪২৯৬; আবূ দাউদ, হা/২৮৬৪)।&lt;br&gt;&lt;br&gt;
+উপরোল্লেখিত হাদীছসমূহ হতে বুঝা যায় যে, খাদ্যের দোষ-ত্রুটি বর্ণনা করা যাবে না। খাবার ভালো লাগলে খেতে হবে, না লাগলে রেখে দিতে হবে। আল্লাহর সন্তুষ্টির উদ্দেশ্যে স্ত্রীর মুখে তুলে দেওয়া খাদ্যের বিনিময়েও আল্লাহ ছাওয়াব দান করবেন। এগুলো স্ত্রীকে ভালোবাসার বাস্তব পদক্ষেপ。&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: قَالَ رَسُولُ اللهِ اللهُ أَكْمَلُ الْمُؤْمِنِينَ إِيمَانًا أَحْسَنُهُمْ خُلُقًا وَخِيَارُكُمْ خِيَارُكُمْ لِنِسَائِهِمْ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবু হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'পূর্ণাঙ্গ ঈমানদার হল সেই ব্যক্তি, যার চরিত্র সর্বাধিক সুন্দর। তোমাদের মধ্যে সর্বোত্তম ব্যক্তি সে যে স্ত্রীদের নিকট উত্তম' (তিরমিযী, হা/১১৬২; মিশকাত হা/৩২৬৪)।&lt;br&gt;&lt;br&gt;
+তাই স্ত্রীদের নিকটে উত্তম হওয়ার জন্য শরী'আত সম্মত পন্থায় চেষ্টা করতে হবে। তাদেরকে হেফাযত করার চেষ্টা করতে হবে। যাতে তারা অন্য পুরুষের সাথে মেলামেশা করতে না পারে, পর্দাহীনভাবে চলাফেরা করতে না পারে。&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنِ الْمُغِيرَةِ قَالَ سَعْدُ بْنُ عُبَادَةَ لَوْ رَأَيْتُ رَجُلاً مَعَ امْرَأَتِي لَضَرَبْتُهُ بِالسَّيْفِ غَيْرَ مُصْفِحٍ، فَقَالَ النَّبِيُّ ﷺ أَتَعْجَبُونَ مِنْ غَيْرَةِ سَعْدٍ، لَأَنَا أَغْيَرُ مِنْهُ وَاللَّهُ أَغْيَرُ مِنِّى».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+মুগীরা (রাঃ) হতে বর্ণিত, সা'দ ইবনু উবাদা (রাঃ) বলেন, আমি যদি অন্য কোনো পুরুষকে আমার স্ত্রীর সাথে দেখতে পাই, তাহলে আমি তাকে তরবারীর ধারালো দিক দিয়ে আঘাত করবো। অর্থাৎ হত্যা করবো। নবী (ﷺ) বললেন, তোমরা কি সা'দের আত্মমর্যাদাবোধের কারণে আশ্চর্যান্বিত হচ্ছো? আমার আত্মমর্যাদাবোধ তার চেয়েও অনেক অধিক এবং আল্লাহর আত্মমর্যাদাবোধ আমার চেয়েও অনেক বেশি (ছহীহ বুখারী, হা/৫২২০; ছহীহ মুসলিম, হা/৩৭৩৭; মিশকাত, হা/৩৩০৯)।&lt;br&gt;&lt;br&gt;
+ইসলাম নারীকে পর্দার অভ্যন্তরে রেখে তার ইজ্জতকে হেফাযত করার ব্যবস্থা করেছে। কিন্তু বর্তমান সমাজের অধিকাংশ লোক স্বীয় স্ত্রী-কন্যাদের বেপর্দায় ছেড়ে দেয়, অন্য পুরুষের সাথে অবাধে মেলামেশার সুযোগ দেয়। এগুলোকে তারা প্রগতি বলে মনে করে। এর সাথে যোগ দিয়েছে তথাকথিত নারী স্বাধীনতার দাবীদার কিছু মহিলা। যারা নারীকে ঘর থেকে বাইরে বের করে আনতে প্রাণান্ত চেষ্টা অব্যাহত রেখেছে। যার বিষাক্ত ফল হচ্ছে নারী নির্যাতন, ইভটিজিং, ধর্ষণ, অপহরণ, এসিড সন্ত্রাস, পরকীয়া, যৌতুক ইত্যাদি। এরপরও তারা নারীকে উলঙ্গ করতে ব্যস্ত। অথচ ইসলাম নারীর ব্যক্তিগত, পারিবারিক, সামাজিক, আর্থিক, সার্বিক নিরাপত্তা বিধান করেছে। নারীর অর্থনৈতিক নিরাপত্তা বিধানের জন্য বিবাহের সময় তার মহরকে বাধ্যতামূলক করেছে (ছহীহ বুখারী, হা/৪৭৭০)। আল্লাহ তাআলা বলেন, 'তোমরা তোমাদের স্ত্রীদের মহর সন্তুষ্টচিত্তে পরিশোধ করো' (নিসা, ৪)।&lt;br&gt;&lt;br&gt;&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>আমানত রক্ষাকারী</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>আমানত রক্ষাকারী</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>&lt;div class="page-text"&gt;&lt;br&gt;আমানত একটি গুরুত্বপূর্ণ বিষয়। যা রক্ষা করা প্রত্যেক মুমিনের উপর আবশ্যিক করা হয়েছে। আমানতের খিয়ানতকারীকে ঈমানহীন বলা হয়েছে। সেজন্য প্রত্যেককে আমানত রক্ষা করে চলতে হবে। খিয়ানতকারীর জন্য পরকালে কঠিন শাস্তি রয়েছে। আল্লাহ বলেন,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;يَا أَيُّهَا الَّذِينَ آمَنُوا لَا تَخُونُوا اللهَ وَالرَّسُوْلَ وَتَخَوْنُوْا أَمَانَاتِكُمْ وَأَنْتُمْ تَعْلَمُوْنَ)&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+'হে ঈমানদারগণ! তোমরা জেনে শুনে আল্লাহ এবং তাঁর রাসূলের সাথে খিয়ানাত করো না এবং নিজেদের আমানাতের খিয়ানাত করো না' (আনফাল, ২৭)।&lt;br&gt;&lt;br&gt;
+খিয়ানত দুই প্রকার : ১. আল্লাহ ও তাঁর রাসূলের সাথে। অর্থাৎ আল্লাহ ও রাসূলের বিধান অমান্য করার মাধ্যমে খিয়ানত। ২. মানুষের গচ্ছিত সম্পদ ভক্ষণ করা কিংবা রক্ষিত জিনিস বিনষ্ট করার মাধ্যমে খিয়ানত করা। এ উভয় প্রকার খিয়ানত হতে বেঁচে থাকা আবশ্যক। অপর একটি আয়াতে আল্লাহ আরো বলেন,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;إِنَّ اللَّهَ يَأْمُرُكُمْ أَنْ تُؤَدُّوا الْأَمَانَاتِ إِلَى أَهْلِهَا )&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+'আল্লাহ তোমাদের আদেশ করেছেন মালিকের নিকটে আমানত পৌঁছে দেওয়ার জন্য' (নিসা, ৫৮)।&lt;br&gt;&lt;br&gt;
+হাদীছে এসেছে,&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ عَدِيِّ بْنِ عَمِيرَةَ قَالَ: قَالَ رَسُولُ اللهِ : مَنِ اسْتَعْمَلْنَاهُ مِنْكُمْ عَلَى عَمَلٍ فَكَتَمَنَا مِخْيَطًا فَمَا فَوْقَهُ كَانَ غُلُوْلاً يَأْتِي بِهِ يَوْمَ الْقِيَامَةِ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;আদী ইবনু আমীরা (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'তোমাদের মধ্যে আমি যাকে কোনো কর্মে নিযুক্ত করি, আর সে আমাদের নিকট হতে একটি সুঁচ অথবা তদাপেক্ষা ছোট কিছু গোপন করে, তা আমানতের খিয়ানত বলে বিবেচিত হবে এবং সে কিয়ামতের দিন তা নিয়ে হাযির হবে' (ছহীহ মুসলিম, হা/৪৮৪৮; মুসনাদে আহমাদ, হা/১৭৭৫৯; মিশকাত, হা/১৭৮০)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي حُمَيْدٍ السَّاعِدِي قَالَ: اسْتَعْمَلَ النَّبِيُّ ﷺ رَجُلًا مِنَ الْأَزْدِ يُقَالُ لَهُ ابْنُ اللُّتْبِيَّةِ عَلَى الصَّدَقَةِ، فَلَمَّا قَدِمَ قَالَ: هَذَا لَكُمْ، وَهَذَا أُهْدِيَ لِي. فَخَطَبَ النَّبِيُّ ﷺ فَحَمِدَ اللَّهَ وَأَثْنَى عَلَيْهِ، ثُمَّ قَالَ: أَمَّا بَعْدُ، فَإِنِّي أَسْتَعْمِلُ رِجَالًا مِنْكُمْ عَلَى أُمُورٍ مِمَّا وَلَا نِي اللهُ، فَيَأْتِي أَحَدُهُمْ فَيَقُولُ: هَذَا لَكُمْ وَهَذِهِ هَدِيَّةٌ أُهْدِيَتْ لِي، فَهَلَّا جَلَسَ فِي بَيْتِ أَبِيهِ أَوْ بَيْتِ أُمِّهِ فَيَنْظُرُ أَيُهْدَى لَهُ أَمْ لَا ، وَالَّذِي نَفْسِي بِيَدِهِ، لَا يَأْخُذُ أَحَدٌ مِنْهُ شَيْئًا إِلَّا جَاءَ بِهِ يَوْمَ الْقِيَامَةِ يَحْمِلُهُ عَلَى رَقَبَتِهِ إِنْ كَانَ بَعِيرًا لَهُ رُغَاءُ، أَوْ بَقْرًا لَهُ خُوَارٌ ، أَوْ شَاةً تَيْعِرُ، ثُمَّ رَفَعَ يَدَيْهُ حَتَّى رَأَيْنَا عُفْرَةَ إِبْطَيْهِ ثُمَّ قَالَ : اللهُمَّ هَلْ بَلَّغْتُ، اللهُمَّ هَلْ بَلَّغْتُ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ হুমায়েদ আস-সায়েদী (রাঃ) হতে বর্ণিত, তিনি বলেন, একবার নবী (ﷺ) ইবনুল লুতবিয়া নামক আযদ গোত্রের এক ব্যক্তিকে যাকাত আদায়ের জন্য নিযুক্ত করলেন। যখন সে যাকাত নিয়ে মদীনায় ফিরলো, তখন বলল, এই অংশ আপনাদের প্রাপ্য যাকাত আর এই অংশ আমাকে হাদিয়া দেওয়া হয়েছে। একথা শুনে নবী ভাষণ দানের জন্য দাঁড়ালেন এবং প্রথমে আল্লাহর গুণগান করে বললেন, ব্যাপার এই যে, আমি তোমাদের মধ্য থেকে কোনো কোনো ব্যক্তিকে সে সকল কাজের জন্য কর্মচারী হিসাবে নিযুক্ত করি। যে সকল কাজের দায়িত্ব আল্লাহ আমার প্রতি সোপর্দ করেছেন। অতঃপর তোমাদের সে ব্যক্তি ফিরে এসে বলে যে, এটা আপনাদের প্রাপ্য যাকাত এবং এটা আমাকে হাদিয়া দেওয়া হয়েছে। সে কেন তার বাপ মায়ের ঘরে বসে দেখল না যে, তাকে হাদিয়া দেওয়া হয় কি-না? আল্লাহর কসম! যে ব্যক্তি এর কোনো কিছু তসরুফ করবে, সে নিশ্চয়ই কিয়ামতের দিন তা আপন ঘাড়ে বহন করে হাযির হবে। যদি তা উট হয়, তাহলে গরগর শব্দ করবে, যদি গরু হয় তাহলে হাম্বা হাম্বা করবে আর যদি ছাগল-ভেড়া হয় তাহলে ভ্যাঁ ভ্যাঁ শব্দ করবে। অতঃপর তিনি তার হস্তদ্বয়কে এমনভাবে উঁচু করলেন, আমরা তাঁর বগলের শুভ্রতা দেখে ফেললাম এবং দুবার বললেন, হে আল্লাহ! আমি কি (তোমার বাণী) পৌঁছে দিয়েছি? (ছহীহ বুখারী, হা/২৫৯৭; ছহীহ মুসলিম, হা/৪৮৪৩; আবু দাউদ, হা/২৯৪৬)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَنَسٍ ، قَالَ : قَلَّمَا خَطَبَنَا رَسُولُ اللهِ ﷺ إِلَّا قَالَ: «لَا إِيمَانَ لِمَنْ لَا أَمَانَةَ لَهُ، وَلَا دِينَ لِمَنْ لَا عَهْدَ لَهُ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আমাদেরকে আনাস (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) প্রায় খুৎবাতে বলতেন, 'যার আমানত নেই তার ঈমান নেই। যার অঙ্গীকার নেই তার ধর্ম নেই' (মুসনাদে আহমাদ, হা/১২৭১৮; ছহীহ ইবনু হিব্বান হা/১৯৪; মিশকাত, হা/৩৫)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي أُمَامَةَ هِ قَالَ: قَالَ رَسُولُ : مَنِ اقْتَطَعَ حَقَّ امْرِئٍ مُسْلِمٍ بِيَمِينِهِ؛ فَقَدْ أَوْجَبَ اللهُ لَهُ النَّارَ، وَحَرَّمَ اللهُ عَلَيْهِ الْجَنَّةَ. فَقَالَ لَهُ رَجُلٌ: وَإِنْ كَانَ شَيْئًا يَسِيرًا يَا رَسُولَ اللَّهِ؟ قَالَ: وَإِنْ كَانَ قَضِيبًا مِنْ أَرَاكِ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবু উমামা (রাঃ) হতে বর্ণিত, তিনি বলেন, রাসূলুল্লাহ (ﷺ) বলেছেন, 'মিথ্যা শপথ করে যে ব্যক্তি কোনো মুসলমানের হক্ক আত্মসাৎ করবে, আল্লাহ তাআলা তার জন্য জাহান্নাম অবধারিত করে রেখেছেন এবং জান্নাত হারাম করেছেন। এক ব্যক্তি তাকে বলল, হে আল্লাহর রাসূল! যদি সামান্য বস্তুও হয়? তিনি বললেন, পিলু গাছের একটি ডালই হোক না কেন' (ছহীহ মুসলিম, হা/৩৭০; ইবনু মাজাহ, হা/২৩২৪; নাসাঈ, হা/৫৪১৯)।&lt;br&gt;&lt;br&gt;
+এই হাদীছ বুঝা যায় যে, কোনো ব্যক্তি যদি, সামান্য জিনিসও আত্মসাৎ করে থাকে, তাহলে তার জন্য, জান্নাত হারাম এবং জাহান্নাম অবধারিত। সুতরাং আত্মসাৎ করা কোনো আদর্শ পুরুষের কাজ নয়। প্রত্যেক নারী- পুরুষের জন্য আত্মসাৎ পরিহার করা অবশ্য কর্তব্য。&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: «قَامَ فِينَا رَسُولُ اللهِ اللهِ ذَاتَ يَوْمٍ، فَذَكَرَ الْغُلُولَ، فَعَظَمَهُ وَعَظَمَ أَمْرَهُ، ثُمَّ قَالَ: لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْمَ الْقِيَامَةِ عَلَى رَقَبَتِهِ بَعِيرُ لَهُ رُغَاءُ يَقُولُ: يَا رَسُولَ اللهِ! أَغِثْنِي، فَأَقُولُ لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ. لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْمَ الْقِيَامَةِ عَلَى رَقَبَتِهِ فُرْسُ لَهُ حَمْحَمَةٌ، فَيَقُولُ: يَا رَسُولَ اللهِ أَغِثْنِي، فَأَقُولُ: لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ، لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْمَ الْقِيَامَةِ عَلَى رَقَبَتِهِ شَاةٌ لَهَا ثُغَاءُ يَقُولُ: يَا رَسُولَ اللَّهِ! أَغِثْنِي، فَأَقُولُ: لَا أَمْلِكُ لَكَ شَيْئًا قَدْ أَبْلَغْتُكَ. لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ الْقِيَامَةِ عَلَى رَقَبَتِهِ نَفْسٌ لَهَا صِيَاحٌ، فَيَقُولُ: يَا رَسُولَ اللهِ أَغِثْنِي، فَأَقُولُ: لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ. لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْمَ الْقِيَامَةِ عَلَى رَقَبَتِهِ رِقَاعٌ تَخْفُقُ، فَيَقُولُ: يَا رَسُولَ اللَّهِ أَغِثْنِي، فَأَقُولُ: لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ. لَا أُلْفِيَنَّ أَحَدَكُمْ يَجِيءُ يَوْمَ الْقِيَامَةِ عَلَى رَقَبَتِهِ صَامِتُ، فَيَقُولُ : يَا رَسُولَ اللهِ! أَغِثْنِي، فَأَقُولُ: لَا أَمْلِكُ لَكَ شَيْئًا، قَدْ أَبْلَغْتُكَ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;আবু হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, একদা রাসূলুল্লাহ (ﷺ) আমাদের মাঝে দাঁড়িয়ে গনীমতের মালে খেয়ানত করা যে জঘন্যতম অপরাধ এবং এর পরিণাম যে অত্যন্ত ভয়াবহ, এ সম্পর্কে আলোচনা করার পর সতর্কবাণী উচ্চারণ করে বললেন, কিয়ামতের দিন আমি তোমাদের কাউকে যেন এই অবস্থায় দেখতে না পাই যে, সে স্বীয় কাঁধের উপর একটি চিৎকাররত উট বহন করে আসবে, আর সে আমাকে লক্ষ্য করে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আর আমি বলব, আজ আমি তোমার জন্য কিছুই করতে পারবো না। আমি তো তোমাকে আল্লাহর বিধান আগেই (দুনিয়াতে) জানিয়ে দিয়েছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এ অবস্থায় দেখতে না পাই যে, সে কাঁধের উপর একটি চিৎকাররত ঘোড়া বহন করে আসবে। আর সে আমাকে লক্ষ্য করে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আর আমি বলব, আজ আমি তোমার জন্য কিছুই করতে পারবো না। আমি তো তোমাকে আল্লাহর বিধান আগেই (দুনিয়াতে) জানিয়ে দিয়েছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এ অবস্থায় দেখতে না পাই যে, সে কাঁধের উপর একটি চিৎকাররত বকরী বহন করে আসবে। আর সে আমাকে লক্ষ্য করে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আর আমি বলবো, আজ আমি তোমার জন্য কিছুই করতে পারবো না। আমি তো তোমাকে আল্লাহর বিধান আগেই (দুনিয়াতে) জানিয়ে দিয়েছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এ অবস্থায় দেখতে না পাই যে, সে কাঁধের উপর একটি চিৎকাররত মানুষকে বহন করে আসবে। আর সে আমাকে লক্ষ্য করে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আর আমি বলব, আজ আমি তোমার জন্য কিছুই করতে পারবো না। আমি তো তোমাকে আল্লাহর বিধান আগেই (দুনিয়াতে) জানিয়ে দিয়েছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এ অবস্থায় দেখতে না পাই যে, সে কাঁধের উপর এলোমেলো কাপড় চোপড় বহন করে আসবে। আর তা তার ঘাড়ের উপর দুলছে। তখন সে আমাকে লক্ষ্য করে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আমি বলব, আজ আমি তোমার জন্য কিছুই করতে পারবো না। আমি তো তোমাকে আল্লাহর বিধান আগেই (দুনিয়াতে) জানিয়ে দিয়েছি। কিয়ামতের দিন আমি যেন তোমাদের কাউকে এমন অবস্থায় দেখতে না পাই যে, সে কাঁধের উপর একটি জড়ো সম্পদ (সোনা-চাঁদি ইত্যাদি) বহন করে আসবে। আর সে আমাকে লক্ষ্য করে বলবে, হে আল্লাহর রাসূল! আমাকে সাহায্য করুন। আর আমি বলব, আজ আমি তোমার জন্য কিছুই করতে পারবো না। আমি তো তোমাকে আল্লাহর&lt;br&gt;&lt;br&gt;বিধান আগেই (দুনিয়াতে) জানিয়ে দিয়েছি (ছহীহ বুখারী, হা/৩০৭৩; ছহীহ মুসলিম, হা/৪৮৩৯; মিশকাত, হা/৩৯৯৬)।&lt;br&gt;&lt;br&gt;&lt;div class="arabic-text"&gt;عَنْ أَبِي هُرَيْرَةَ قَالَ: «أَهْدَى رَجُلٌ لِرَسُولِ اللهِ ﷺ غُلَامًا يُقَالُ لَهُ: مِدْعَمُ فَبَيْنَمَا مِدْعَمُ يَحُطُّ رَحْلًا لِرَسُولِ اللهِ ﷺ إِذْ أَصَابَهُ سَهُمْ عَائِرٌ فَقَتَلَهُ، فَقَالَ النَّاسُ: هَنِيئًا لَهُ الْجَنَّةُ، فَقَالَ رَسُولُ اللهِ ﷺ: كَلَّا ، وَالَّذِي نَفْسِي بِيَدِهِ إِنَّ الشَّمْلَةَ الَّتِي أَخَذَهَا يَوْمَ خَيْبَرَ مِنَ الْمَغَانِمِ لَمْ تُصِبْهَا الْمَقَاسِمُ، لَتَشْتَعِلُ عَلَيْهِ نَارًا . فَلَمَّا سَمِعَ ذَلِكَ النَّاسُ جَاءَ رَجُلٌ بِشِرَاكٍ، أَوْ شِرَاكَيْنِ إِلَى النَّبِيِّ ﷺ فَقَالَ: شِرَاكَ مِنْ نَارٍ، أَوْ شِرَاكَانِ مِنْ نَارٍ».&lt;/div&gt;&lt;br&gt;&lt;br&gt;
+আবূ হুরায়রা (রাঃ) হতে বর্ণিত, তিনি বলেন, এক ব্যক্তি রাসূলুল্লাহ (ﷺ)-কে একটি গোলাম হাদিয়া দিয়েছিল, যার নাম মিদআম। এক সময় মিদআম রাসূলুল্লাহ (ﷺ)-এর বাহন প্রস্তুত করছিল। হঠাৎ অজ্ঞাত তীর এসে তার গায়ে লাগল এবং তীর তাকে নিহত করলো। লোকেরা বলল, তার জন্য জান্নাতের সুসংবাদ। রাসূলুল্লাহ (ﷺ) বললেন, কখনো নয়। আল্লাহর কসম! সে খায়বরের দিন দশের সম্পদ হতে একটি চাদর আত্মসাৎ করেছিল। এ চাদর জাহান্নামের আগুনকে তার উপর ক্ষিপ্ত করবে। লোকেরা একথা শুনলো এবং এক ব্যক্তি একটি জুতার ফিতা বা দুটি জুতার ফিতা নিয়ে নবী (ﷺ)-এর নিকট আসলো। ফলে তিনি বললেন, একটি জুতার ফিতা বা দুটি জুতার ফিতার সমান জিনিস আত্মসাৎ করলেও তার জন্য জাহান্নাম' (ছহীহ বুখারী, হা/৪২৩৪; ছহীহ মুসলিম, হা/৩২৫; মিশকাত, হা/৩৯৯৭)।&lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>